<commit_message>
Testing with different positions
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inbetgroup-my.sharepoint.com/personal/adriana_koleva_inbet_com/Documents/Projects/GitHub/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="168" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A49DEBEC-6564-4E2D-9A15-7F3E3CA8D9B8}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA513391-7D14-45F0-B3FA-87DF8D711B70}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Position</t>
   </si>
@@ -45,22 +45,7 @@
     <t>HR Director</t>
   </si>
   <si>
-    <t>Affiliate Director</t>
-  </si>
-  <si>
-    <t>CRM Director</t>
-  </si>
-  <si>
-    <t>CRM / Retention</t>
-  </si>
-  <si>
     <t>HR</t>
-  </si>
-  <si>
-    <t>Affiliate</t>
-  </si>
-  <si>
-    <t>Директор на CRM стратегията – задържане на играчи, бонус програми, жизнен цикъл на клиента.</t>
   </si>
   <si>
     <t>HR директорът ръководи пълния спектър от човешки ресурси за inbet Group, обхващайки привличането на таланти, възнагражденията, обучението и развитието, съответствието с човешките изисквания и организационния дизайн на всички пазари.</t>
@@ -81,54 +66,10 @@
 Владеене на английски език; допълнителни езици са плюс."</t>
   </si>
   <si>
-    <t>Директорът на афилиейт отдела отговаря за стратегията за афилиейт и партньорски канали на всички пазари за залози, като стимулира привличането на играчи чрез афилиейт мрежи, медийни партньори и инфлуенсъри във вертикала на казино залаганията.</t>
-  </si>
-  <si>
-    <t>Дефиниране на глобалната партньорска стратегия, структурите на комисионните и рамките на партньорските нива.
-Набиране, договаряне и управление на взаимоотношения с водещи партньори в спортните залози и онлайн казината.
-Надзор на операциите на партньорската платформа (проследяване, отчитане, предотвратяване на измами).
-Определяне на ключови показатели за ефективност (KPI) за CPA, дял от приходите и хибридни сделки; наблюдение на възвръщаемостта на инвестициите по пазари.
-Сътрудничество с маркетинг и CRM за съгласуване на партньорските промоции с кампаниите за жизнения цикъл на играчите.
-Осигуряване на съответствие между партньорските дейности и рекламните стандарти и разпоредбите за хазарта в съответната юрисдикция.
-Ръководство и развитие на екипа на партньорите.</t>
-  </si>
-  <si>
-    <t>5+ години опит в афилиейт маркетинга в iGaming индустрията.
-Разширена мрежа от афилиейт партньори за казина/спортни залагания в Източна Европа и Латинска Америка.
-Владеене на афилиейт платформи (Income Access, Cellxpert или еквивалентни).
-Основано на данни; увереност в кохортния анализ и LTV моделирането.
-Владеене на английски език.</t>
-  </si>
-  <si>
     <t>Salary range min</t>
   </si>
   <si>
     <t>Salary range max</t>
-  </si>
-  <si>
-    <t>test</t>
-  </si>
-  <si>
-    <t>CRM Manager</t>
-  </si>
-  <si>
-    <t>CRM мениджърът превръща стратегията на CRM директора в изпълнени кампании и автоматизирани процеси, управлявайки ежедневните операции по задържане на играчите на inbet.</t>
-  </si>
-  <si>
-    <t>Планирайте и изпълнявайте многоканални CRM кампании (имейл, SMS, push, в приложения) за казино и спортни залагания.
-Изграждайте и оптимизирайте сегментирането на играчите и потоците за автоматизация на жизнения цикъл.
-Управлявайте промоционални календари, съобразени със спортни събития и пускане на казино игри.
-Наблюдавайте ефективността на кампаниите и оптимизирайте съответно.
-Координирайте се с екипите за креативност, продукти и плащания за безпроблемно преживяване на играчите.
-Надзор на CRM експертите и предоставяйте коучинг.
-Осигурете съответствие на всички комуникации с разпоредбите за реклама на хазарт.</t>
-  </si>
-  <si>
-    <t>3+ години опит в управлението на CRM в iGaming.
-Владее инструменти за автоматизация на CRM и платформи за клиентски данни.
-Силно разбиране на динамиката на продуктите за казино и спортни залози.
-Аналитично мислене с опит в A/B тестване.
-Владее свободно английски език.</t>
   </si>
 </sst>
 </file>
@@ -184,16 +125,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -210,7 +148,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -491,26 +428,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="7" customWidth="1"/>
-    <col min="3" max="3" width="55.77734375" style="7" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="6" customWidth="1"/>
+    <col min="3" max="3" width="55.77734375" style="6" customWidth="1"/>
     <col min="4" max="4" width="27.88671875" customWidth="1"/>
     <col min="5" max="5" width="24.6640625" customWidth="1"/>
-    <col min="6" max="6" width="26.44140625" style="7" customWidth="1"/>
-    <col min="7" max="7" width="19.77734375" style="7" customWidth="1"/>
+    <col min="6" max="6" width="26.44140625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="19.77734375" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -519,322 +456,223 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>19</v>
+      <c r="F1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="7">
+      <c r="F2" s="6">
         <v>2500</v>
       </c>
-      <c r="G2" s="7">
+      <c r="G2" s="6">
         <v>3500</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F3" s="7">
-        <v>2500</v>
-      </c>
-      <c r="G3" s="7">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="409.6" x14ac:dyDescent="0.35">
-      <c r="A5" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" s="7">
-        <v>2000</v>
-      </c>
-      <c r="G5" s="7">
-        <v>3000</v>
-      </c>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
-      <c r="B30" s="4"/>
-      <c r="C30" s="4"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
-      <c r="B32" s="4"/>
-      <c r="C32" s="4"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
-      <c r="B34" s="4"/>
-      <c r="C34" s="4"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
-      <c r="B35" s="4"/>
-      <c r="C35" s="4"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
-      <c r="B36" s="4"/>
-      <c r="C36" s="4"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="2"/>
-      <c r="B38" s="4"/>
-      <c r="C38" s="4"/>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="2"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
+      <c r="C38" s="3"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="2"/>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4"/>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="2"/>
-      <c r="B41" s="4"/>
-      <c r="C41" s="4"/>
+      <c r="C40" s="3"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="2"/>
-      <c r="B42" s="4"/>
-      <c r="C42" s="4"/>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="2"/>
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
+      <c r="C42" s="3"/>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="2"/>
-      <c r="B44" s="4"/>
-      <c r="C44" s="4"/>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="2"/>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C47" s="4"/>
-    </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C49" s="4"/>
-    </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C51" s="4"/>
-    </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C53" s="4"/>
-    </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C55" s="4"/>
-    </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B89" s="4"/>
+      <c r="C44" s="3"/>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C46" s="3"/>
+    </row>
+    <row r="80" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B80" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Testing with 0 available positions.
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inbetgroup-my.sharepoint.com/personal/adriana_koleva_inbet_com/Documents/Projects/GitHub/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CA513391-7D14-45F0-B3FA-87DF8D711B70}"/>
+  <xr:revisionPtr revIDLastSave="171" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{815D2EA9-6D3D-4B37-8691-0FC27D80B3DD}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Position</t>
   </si>
@@ -42,30 +42,6 @@
     <t>Requirements</t>
   </si>
   <si>
-    <t>HR Director</t>
-  </si>
-  <si>
-    <t>HR</t>
-  </si>
-  <si>
-    <t>HR директорът ръководи пълния спектър от човешки ресурси за inbet Group, обхващайки привличането на таланти, възнагражденията, обучението и развитието, съответствието с човешките изисквания и организационния дизайн на всички пазари.</t>
-  </si>
-  <si>
-    <t>„Определяне и изпълнение на груповата HR стратегия, съобразена с плана за растеж на бизнеса с казино залагания.
-Надзор на процесите за набиране на персонал за всички пазари (BG, MX, UZ, PE, AL).
-Проектиране и поддържане на рамки за възнаграждения и обезщетения, конкурентни в рамките на iGaming индустрията.
-Управление на циклите на управление на производителността, планиране на наследяване и програми за развитие на лидерските качества.
-Осигуряване на спазване на изискванията на трудовото законодателство във всички оперативни юрисдикции.
-Партниране с COO и главните изпълнителни директори по организационния дизайн и планирането на персонала.
-Подкрепа за фирмената култура, ангажираността и задържането на служителите.“</t>
-  </si>
-  <si>
-    <t>"7+ години опит в областта на човешките ресурси, с поне 3 години на директорско ниво в iGaming, финтех или технологични компании.
-Доказан опит в изграждането на HR функции в организации с множество държави.
-Силни познания по българското трудово законодателство; опитът в областта на човешките ресурси в сектора на игрите е предимство.
-Владеене на английски език; допълнителни езици са плюс."</t>
-  </si>
-  <si>
     <t>Salary range min</t>
   </si>
   <si>
@@ -76,7 +52,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,12 +67,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF292A2E"/>
-      <name val="Segoe UI"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -125,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -139,14 +109,8 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -428,16 +392,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="6" customWidth="1"/>
-    <col min="3" max="3" width="55.77734375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="5" customWidth="1"/>
+    <col min="3" max="3" width="55.77734375" style="5" customWidth="1"/>
     <col min="4" max="4" width="27.88671875" customWidth="1"/>
     <col min="5" max="5" width="24.6640625" customWidth="1"/>
-    <col min="6" max="6" width="26.44140625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="19.77734375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="26.44140625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="19.77734375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
@@ -457,34 +421,16 @@
         <v>4</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="6">
-        <v>2500</v>
-      </c>
-      <c r="G2" s="6">
-        <v>3500</v>
-      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2"/>
@@ -656,23 +602,48 @@
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
     </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="2"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+    </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="2"/>
+      <c r="B38" s="3"/>
       <c r="C38" s="3"/>
     </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="2"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+    </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="2"/>
+      <c r="B40" s="3"/>
       <c r="C40" s="3"/>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C42" s="3"/>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C44" s="3"/>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C46" s="3"/>
-    </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B80" s="3"/>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="2"/>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C43" s="3"/>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C45" s="3"/>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C47" s="3"/>
+    </row>
+    <row r="49" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C49" s="3"/>
+    </row>
+    <row r="51" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C51" s="3"/>
+    </row>
+    <row r="85" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B85" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
FINAL - Ready to use
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inbetgroup-my.sharepoint.com/personal/adriana_koleva_inbet_com/Documents/Projects/GitHub/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="171" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{815D2EA9-6D3D-4B37-8691-0FC27D80B3DD}"/>
+  <xr:revisionPtr revIDLastSave="170" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FB51BD5-F724-4CA7-BE92-9B7915B7D585}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="2232" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>Position</t>
   </si>
@@ -42,17 +42,100 @@
     <t>Requirements</t>
   </si>
   <si>
+    <t>HR Director</t>
+  </si>
+  <si>
+    <t>Affiliate Director</t>
+  </si>
+  <si>
+    <t>CRM Director</t>
+  </si>
+  <si>
+    <t>CRM / Retention</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>Affiliate</t>
+  </si>
+  <si>
+    <t>Директор на CRM стратегията – задържане на играчи, бонус програми, жизнен цикъл на клиента.</t>
+  </si>
+  <si>
+    <t>HR директорът ръководи пълния спектър от човешки ресурси за inbet Group, обхващайки привличането на таланти, възнагражденията, обучението и развитието, съответствието с човешките изисквания и организационния дизайн на всички пазари.</t>
+  </si>
+  <si>
+    <t>„Определяне и изпълнение на груповата HR стратегия, съобразена с плана за растеж на бизнеса с казино залагания.
+Надзор на процесите за набиране на персонал за всички пазари (BG, MX, UZ, PE, AL).
+Проектиране и поддържане на рамки за възнаграждения и обезщетения, конкурентни в рамките на iGaming индустрията.
+Управление на циклите на управление на производителността, планиране на наследяване и програми за развитие на лидерските качества.
+Осигуряване на спазване на изискванията на трудовото законодателство във всички оперативни юрисдикции.
+Партниране с COO и главните изпълнителни директори по организационния дизайн и планирането на персонала.
+Подкрепа за фирмената култура, ангажираността и задържането на служителите.“</t>
+  </si>
+  <si>
+    <t>"7+ години опит в областта на човешките ресурси, с поне 3 години на директорско ниво в iGaming, финтех или технологични компании.
+Доказан опит в изграждането на HR функции в организации с множество държави.
+Силни познания по българското трудово законодателство; опитът в областта на човешките ресурси в сектора на игрите е предимство.
+Владеене на английски език; допълнителни езици са плюс."</t>
+  </si>
+  <si>
+    <t>Директорът на афилиейт отдела отговаря за стратегията за афилиейт и партньорски канали на всички пазари за залози, като стимулира привличането на играчи чрез афилиейт мрежи, медийни партньори и инфлуенсъри във вертикала на казино залаганията.</t>
+  </si>
+  <si>
+    <t>Дефиниране на глобалната партньорска стратегия, структурите на комисионните и рамките на партньорските нива.
+Набиране, договаряне и управление на взаимоотношения с водещи партньори в спортните залози и онлайн казината.
+Надзор на операциите на партньорската платформа (проследяване, отчитане, предотвратяване на измами).
+Определяне на ключови показатели за ефективност (KPI) за CPA, дял от приходите и хибридни сделки; наблюдение на възвръщаемостта на инвестициите по пазари.
+Сътрудничество с маркетинг и CRM за съгласуване на партньорските промоции с кампаниите за жизнения цикъл на играчите.
+Осигуряване на съответствие между партньорските дейности и рекламните стандарти и разпоредбите за хазарта в съответната юрисдикция.
+Ръководство и развитие на екипа на партньорите.</t>
+  </si>
+  <si>
+    <t>5+ години опит в афилиейт маркетинга в iGaming индустрията.
+Разширена мрежа от афилиейт партньори за казина/спортни залагания в Източна Европа и Латинска Америка.
+Владеене на афилиейт платформи (Income Access, Cellxpert или еквивалентни).
+Основано на данни; увереност в кохортния анализ и LTV моделирането.
+Владеене на английски език.</t>
+  </si>
+  <si>
     <t>Salary range min</t>
   </si>
   <si>
     <t>Salary range max</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>CRM Manager</t>
+  </si>
+  <si>
+    <t>CRM мениджърът превръща стратегията на CRM директора в изпълнени кампании и автоматизирани процеси, управлявайки ежедневните операции по задържане на играчите на inbet.</t>
+  </si>
+  <si>
+    <t>Планирайте и изпълнявайте многоканални CRM кампании (имейл, SMS, push, в приложения) за казино и спортни залагания.
+Изграждайте и оптимизирайте сегментирането на играчите и потоците за автоматизация на жизнения цикъл.
+Управлявайте промоционални календари, съобразени със спортни събития и пускане на казино игри.
+Наблюдавайте ефективността на кампаниите и оптимизирайте съответно.
+Координирайте се с екипите за креативност, продукти и плащания за безпроблемно преживяване на играчите.
+Надзор на CRM експертите и предоставяйте коучинг.
+Осигурете съответствие на всички комуникации с разпоредбите за реклама на хазарт.</t>
+  </si>
+  <si>
+    <t>3+ години опит в управлението на CRM в iGaming.
+Владее инструменти за автоматизация на CRM и платформи за клиентски данни.
+Силно разбиране на динамиката на продуктите за казино и спортни залози.
+Аналитично мислене с опит в A/B тестване.
+Владее свободно английски език.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -67,6 +150,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF292A2E"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -95,7 +184,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -104,14 +193,24 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -392,26 +491,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G85"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5546875" style="5" customWidth="1"/>
-    <col min="3" max="3" width="55.77734375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" style="7" customWidth="1"/>
+    <col min="3" max="3" width="55.77734375" style="7" customWidth="1"/>
     <col min="4" max="4" width="27.88671875" customWidth="1"/>
     <col min="5" max="5" width="24.6640625" customWidth="1"/>
-    <col min="6" max="6" width="26.44140625" style="5" customWidth="1"/>
-    <col min="7" max="7" width="19.77734375" style="5" customWidth="1"/>
+    <col min="6" max="6" width="26.44140625" style="7" customWidth="1"/>
+    <col min="7" max="7" width="19.77734375" style="7" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -420,230 +519,322 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="7">
+        <v>2500</v>
+      </c>
+      <c r="G2" s="7">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" s="7">
+        <v>2500</v>
+      </c>
+      <c r="G3" s="7">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="409.6" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="7">
+        <v>2000</v>
+      </c>
+      <c r="G5" s="7">
+        <v>3000</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="2"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="2"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="2"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="2"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="2"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="2"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="2"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="2"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="2"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="2"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
-      <c r="B40" s="3"/>
-      <c r="C40" s="3"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="2"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C43" s="3"/>
+      <c r="A43" s="2"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="2"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C45" s="3"/>
+      <c r="A45" s="2"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C47" s="3"/>
+      <c r="C47" s="4"/>
     </row>
     <row r="49" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C49" s="3"/>
+      <c r="C49" s="4"/>
     </row>
     <row r="51" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C51" s="3"/>
-    </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B85" s="3"/>
+      <c r="C51" s="4"/>
+    </row>
+    <row r="53" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C53" s="4"/>
+    </row>
+    <row r="55" spans="3:3" x14ac:dyDescent="0.3">
+      <c r="C55" s="4"/>
+    </row>
+    <row r="89" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B89" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Lots of testing for trying to bypass visual studio
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://inbetgroup-my.sharepoint.com/personal/adriana_koleva_inbet_com/Documents/Projects/GitHub/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="170" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FB51BD5-F724-4CA7-BE92-9B7915B7D585}"/>
+  <xr:revisionPtr revIDLastSave="179" documentId="11_F25DC773A252ABDACC1048DD919B7AA85ADE58ED" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B37D7A75-AA66-4F92-B4FB-5D5F055CFD92}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="29">
   <si>
     <t>Position</t>
   </si>
@@ -129,6 +129,27 @@
 Силно разбиране на динамиката на продуктите за казино и спортни залози.
 Аналитично мислене с опит в A/B тестване.
 Владее свободно английски език.</t>
+  </si>
+  <si>
+    <t>CRM Expert</t>
+  </si>
+  <si>
+    <t>The CRM Expert executes player retention campaigns and manages daily CRM operations, supporting the growth of player lifetime value across casino and sports betting segments.</t>
+  </si>
+  <si>
+    <t>Build and send targeted CRM campaigns across email, SMS, push and in-platform channels.
+Create player segments based on behaviour, product preference and activity level.
+Manage bonus and free-spin offers in the bonus engine; ensure correct tracking.
+Monitor campaign results and prepare performance reports.
+Support A/B testing initiatives.
+Maintain compliance with responsible gambling messaging requirements.</t>
+  </si>
+  <si>
+    <t>2+ years in CRM operations, preferably in online casino or sports betting.
+Hands-on with CRM or marketing automation platforms.
+Good understanding of casino game types and sportsbook operations.
+Detail-oriented; comfortable handling large datasets.
+Fluent English.</t>
   </si>
 </sst>
 </file>
@@ -618,10 +639,28 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
+    <row r="6" spans="1:7" ht="288.60000000000002" x14ac:dyDescent="0.35">
+      <c r="A6" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="7">
+        <v>3000</v>
+      </c>
+      <c r="G6" s="7">
+        <v>3100</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>

</xml_diff>